<commit_message>
Updated with first version
</commit_message>
<xml_diff>
--- a/InputData/land/CSpULApYbP/CO2 Sequestered per Unit Land Area per Year by Pol.xlsx
+++ b/InputData/land/CSpULApYbP/CO2 Sequestered per Unit Land Area per Year by Pol.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Indonesia/eps-indonesia-1.2.3.3/InputData/land/CSpULApYbP/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/land/CSpULApYbP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC39E15B-E0D0-964C-9C91-B67B2215740A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E86C1B4-C0BA-8049-8417-26B5E2F3F889}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1079,7 +1079,7 @@
         <v>58</v>
       </c>
       <c r="B14">
-        <v>1197.7</v>
+        <v>197.7</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -1087,7 +1087,7 @@
         <v>59</v>
       </c>
       <c r="B15">
-        <v>1192.7</v>
+        <v>192.7</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -1095,7 +1095,7 @@
         <v>60</v>
       </c>
       <c r="B16">
-        <v>1159.3</v>
+        <v>159.30000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -1103,7 +1103,7 @@
         <v>61</v>
       </c>
       <c r="B17">
-        <v>1263.9000000000001</v>
+        <v>263.89999999999998</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -1111,7 +1111,7 @@
         <v>62</v>
       </c>
       <c r="B18">
-        <v>1201.7</v>
+        <v>201.7</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B19" s="1">
         <f>AVERAGE(B13:B18)</f>
-        <v>1213.55</v>
+        <v>380.21666666666664</v>
       </c>
       <c r="C19" s="1"/>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B23" s="3">
         <f>B19*B21</f>
-        <v>4449.6833333333334</v>
+        <v>1394.1277777777777</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="B26" s="9">
         <f>B23/B25</f>
-        <v>111.24208333333334</v>
+        <v>34.853194444444441</v>
       </c>
     </row>
   </sheetData>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="B3" s="3">
         <f>'Indonesia Data'!B26*grams_per_ton/acres_per_hectare</f>
-        <v>45018143.434302561</v>
+        <v>14104609.1517551</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="B5" s="3">
         <f>'Indonesia Data'!B26*grams_per_ton/acres_per_hectare</f>
-        <v>45018143.434302561</v>
+        <v>14104609.1517551</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>

</xml_diff>

<commit_message>
Updated land-use data with indonesia specific data
</commit_message>
<xml_diff>
--- a/InputData/land/CSpULApYbP/CO2 Sequestered per Unit Land Area per Year by Pol.xlsx
+++ b/InputData/land/CSpULApYbP/CO2 Sequestered per Unit Land Area per Year by Pol.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Postdoc Projects/eps-indonesia-cpl/InputData/land/CSpULApYbP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA26AD71-5EE7-4C4D-8E9D-7E0528084B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CBEEC0-0D42-1C4C-B54F-E09E03608452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21360" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="96">
   <si>
     <t>CSpULApYbP CO2 Sequestered per Unit Land Area per Year by Policy</t>
   </si>
@@ -273,6 +273,63 @@
   </si>
   <si>
     <t>US</t>
+  </si>
+  <si>
+    <t>Peatland</t>
+  </si>
+  <si>
+    <t>https://gggi.org/wp-content/uploads/2020/11/Indonesia-Peat-Insight-Brief_October2020_tentative.pdf</t>
+  </si>
+  <si>
+    <t>Input Carbon (Gt C)</t>
+  </si>
+  <si>
+    <t>CO₂ Equivalent (Gt CO₂)</t>
+  </si>
+  <si>
+    <t>CO₂ Equivalent (t CO₂)</t>
+  </si>
+  <si>
+    <t>Area (Mha)</t>
+  </si>
+  <si>
+    <t>Area (ha)</t>
+  </si>
+  <si>
+    <t>Emissions per ha (t CO₂/ha)</t>
+  </si>
+  <si>
+    <t>0.81 Gt C</t>
+  </si>
+  <si>
+    <t>2.9727 Gt CO₂</t>
+  </si>
+  <si>
+    <t>2,972,700,000 t CO₂</t>
+  </si>
+  <si>
+    <t>0.79 Mha</t>
+  </si>
+  <si>
+    <t>790,000 ha</t>
+  </si>
+  <si>
+    <t>3,763.54 t CO₂/ha</t>
+  </si>
+  <si>
+    <t>2.57 Gt C</t>
+  </si>
+  <si>
+    <t>9.4359 Gt CO₂</t>
+  </si>
+  <si>
+    <t>9,435,900,000 t CO₂</t>
+  </si>
+  <si>
+    <t>11,942.91 t CO₂/ha</t>
+  </si>
+  <si>
+    <t>https://www.nature.com/articles/nature01131</t>
   </si>
 </sst>
 </file>
@@ -355,7 +412,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -378,6 +435,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -995,7 +1053,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="78" customWidth="1"/>
@@ -1034,8 +1092,9 @@
       <c r="A6" t="s">
         <v>41</v>
       </c>
-      <c r="B6">
-        <v>923.1</v>
+      <c r="B6" s="14">
+        <f>11942.91</f>
+        <v>11942.91</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -1060,7 +1119,7 @@
       </c>
       <c r="B9" s="9">
         <f>B6*B7/B8</f>
-        <v>6.9232500000000003</v>
+        <v>89.57182499999999</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -1104,7 +1163,7 @@
         <v>159.30000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>61</v>
       </c>
@@ -1112,7 +1171,7 @@
         <v>263.89999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>62</v>
       </c>
@@ -1120,7 +1179,7 @@
         <v>201.7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>63</v>
       </c>
@@ -1130,12 +1189,12 @@
       </c>
       <c r="C19" s="1"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>56</v>
       </c>
@@ -1144,7 +1203,7 @@
         <v>3.6666666666666665</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>64</v>
       </c>
@@ -1153,7 +1212,7 @@
         <v>783.01666666666654</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>75</v>
       </c>
@@ -1161,7 +1220,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>66</v>
       </c>
@@ -1170,7 +1229,75 @@
         <v>19.575416666666662</v>
       </c>
     </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>85</v>
+      </c>
+      <c r="B30" t="s">
+        <v>86</v>
+      </c>
+      <c r="C30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" t="s">
+        <v>89</v>
+      </c>
+      <c r="F30" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" t="s">
+        <v>92</v>
+      </c>
+      <c r="C31" t="s">
+        <v>93</v>
+      </c>
+      <c r="D31" t="s">
+        <v>88</v>
+      </c>
+      <c r="E31" t="s">
+        <v>89</v>
+      </c>
+      <c r="F31" t="s">
+        <v>94</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A28" r:id="rId1" xr:uid="{680CBD88-707E-5348-91F0-50F88AB8DB5F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1203,7 +1330,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F3C4976-BEA3-4045-A2B2-27FA6ED5BF6A}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -1227,7 +1354,7 @@
       <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="13">
         <v>1746915.2241455801</v>
       </c>
     </row>
@@ -1242,7 +1369,7 @@
       <c r="E3" t="s">
         <v>10</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="13">
         <v>1973063.9059045599</v>
       </c>
     </row>
@@ -1256,7 +1383,7 @@
       <c r="E4" t="s">
         <v>11</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="13">
         <v>0</v>
       </c>
     </row>
@@ -1271,7 +1398,7 @@
       <c r="E5" t="s">
         <v>12</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="13">
         <v>5617477.9584253896</v>
       </c>
     </row>
@@ -1281,12 +1408,12 @@
       </c>
       <c r="B6" s="13">
         <f>('Indonesia Data'!B2+'Indonesia Data'!B9)*grams_per_ton/acres_per_hectare</f>
-        <v>7253293.1344974805</v>
+        <v>40700036.421764024</v>
       </c>
       <c r="E6" t="s">
         <v>13</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="13">
         <v>4936277.0697642304</v>
       </c>
     </row>
@@ -1301,11 +1428,33 @@
       <c r="E7" t="s">
         <v>14</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="13">
         <v>17025923.6378057</v>
       </c>
     </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="13">
+        <v>24266568</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B12" s="13"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B13" s="13"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A10" r:id="rId1" xr:uid="{133676CD-357E-8D4F-956A-7C48A23E3EE0}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1461,7 +1610,7 @@
       </c>
       <c r="B6" s="13">
         <f>Sheet1!B6</f>
-        <v>7253293.1344974805</v>
+        <v>40700036.421764024</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>

</xml_diff>